<commit_message>
eval finetuned model, corrected datenfluss
</commit_message>
<xml_diff>
--- a/Trainingsdaten/Trainingsdaten-KI.xlsx
+++ b/Trainingsdaten/Trainingsdaten-KI.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wpx619\.AAA_Python_MTH\Matching\Trainingsdaten\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8335282C-B99A-4660-9855-33F688A11124}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADA65D2D-29A1-4327-9083-52CC56268E26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="6285" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11030" yWindow="380" windowWidth="16560" windowHeight="20970" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle2" sheetId="1" r:id="rId1"/>
@@ -3811,7 +3811,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -3825,7 +3825,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -3839,7 +3839,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -3853,7 +3853,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -3867,7 +3867,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>2</v>
       </c>
@@ -3881,7 +3881,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>2</v>
       </c>
@@ -3895,7 +3895,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>2</v>
       </c>
@@ -3909,7 +3909,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>2</v>
       </c>
@@ -3923,7 +3923,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>2</v>
       </c>
@@ -3951,7 +3951,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>2</v>
       </c>
@@ -3965,21 +3965,21 @@
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>2</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="2" t="s">
         <v>44</v>
       </c>
       <c r="D13" s="4" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>2</v>
       </c>
@@ -7006,7 +7006,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="230" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A230" t="s">
         <v>1</v>
       </c>
@@ -7020,7 +7020,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="231" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A231" t="s">
         <v>1</v>
       </c>
@@ -7034,7 +7034,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="232" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A232" t="s">
         <v>1</v>
       </c>
@@ -7048,7 +7048,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="233" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A233" t="s">
         <v>1</v>
       </c>
@@ -7062,7 +7062,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="234" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A234" t="s">
         <v>1</v>
       </c>
@@ -7076,7 +7076,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="235" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A235" t="s">
         <v>1</v>
       </c>
@@ -7090,7 +7090,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="236" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A236" t="s">
         <v>1</v>
       </c>
@@ -7104,7 +7104,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="237" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A237" t="s">
         <v>1</v>
       </c>
@@ -7118,7 +7118,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="238" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A238" t="s">
         <v>1</v>
       </c>
@@ -7146,7 +7146,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="240" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A240" t="s">
         <v>1</v>
       </c>
@@ -8080,7 +8080,7 @@
   <autoFilter ref="A1:E305" xr:uid="{00000000-0001-0000-0000-000000000000}">
     <filterColumn colId="0">
       <filters>
-        <filter val="IfcBeam"/>
+        <filter val="IfcSlab"/>
       </filters>
     </filterColumn>
     <filterColumn colId="1">
@@ -8194,6 +8194,7 @@
         <filter val="MOLDING"/>
         <filter val="MOVABLE"/>
         <filter val="MULLION"/>
+        <filter val="NOTDEFINED"/>
         <filter val="OVEREXCAVATION"/>
         <filter val="PAD_FOOTING"/>
         <filter val="PARAPET"/>
@@ -13823,6 +13824,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>